<commit_message>
Improve subject line prompt and regenerate corredoras emails
Enforce max 8-word provocative subjects with urgency. Prohibit
corporate filler words. Add tone examples. Regenerate Excel output.

https://claude.ai/code/session_01DWU7frtt2nZeg1H9Fnsb63
</commit_message>
<xml_diff>
--- a/resility_correos_corredoras.xlsx
+++ b/resility_correos_corredoras.xlsx
@@ -506,7 +506,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RESILITY — Correos de Ventas Personalizados  |  Generado: 12/03/2026 19:35</t>
+          <t>RESILITY — Correos de Ventas Personalizados  |  Generado: 12/03/2026 19:56</t>
         </is>
       </c>
     </row>
@@ -608,16 +608,17 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Beroiza Seguros y la nueva satisfacción regulatoria que la CMF ya está exigiendo</t>
+          <t>¿Quién protege las pólizas de sus clientes hoy?</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
           <t>María Isabel,
-Como corredora de seguros, Beroiza maneja diariamente RUT, datos de salud, pólizas y antecedentes financieros de cientos de clientes. Esa información es exactamente lo que buscan los atacantes, y las corredoras son hoy el eslabón más apuntado de la cadena aseguradora.
-Con la Ley 21.663 ya vigente, la obligación de proteger esos datos y reportar incidentes es directa, con multas de hasta $3.000 millones CLP. Y seamos francos: armar un equipo interno de ciberseguridad no es viable ni necesario para una corredora.
-Resility funciona como tu CyberSOC externalizado: monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio CMF resuelto, sin sumar headcount. Nuestros clientes en el sector reducen un 70% el tiempo de detección de incidentes versus esquemas tradicionales.
-¿Tienes 15 minutos esta semana para mostrarte cómo quedaría protegida Beroiza sin complejidad operativa?
+Las corredoras de seguros son hoy el blanco favorito de los atacantes: manejan RUT, datos de salud, cuentas bancarias y detalles de siniestros de cientos de clientes, y rara vez cuentan con un equipo dedicado de ciberseguridad. Beroiza Seguros no es la excepción en ese perfil de riesgo.
+Con la Ley 21.663 ya vigente, una filtración de datos no solo destruye la confianza de sus asegurados — implica multas de hasta $3.000 millones CLP y la obligación de reportar incidentes ante la CMF.
+Resility actúa como su equipo de ciberseguridad 24/7, sin que necesite contratar ni un solo especialista. Nuestra IA, entrenada en amenazas reales de Latinoamérica, reduce el tiempo de detección de incidentes en un 70% versus un SOC tradicional.
+¿Tiene 15 minutos esta semana para que le muestre qué tan expuesta está su operación hoy y cómo cerramos esas brechas rápidamente?
+Quedo atenta a su respuesta.
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>
@@ -668,17 +669,16 @@
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>Seguros Broker y la nueva Ley de Ciberseguridad: un riesgo que se puede evitar</t>
+          <t>¿Quién protege los datos de sus asegurados hoy?</t>
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>Lily, buenas tardes.
-Las corredoras de seguros como Seguros Broker manejan a diario datos que los atacantes más buscan: RUT, información de salud, pólizas, cuentas bancarias. Y en la mayoría de los casos, no cuentan con un equipo dedicado a protegerlos.
-Con la Ley 21.663 ya vigente, tu empresa está obligada a resguardar esos datos y reportar incidentes, con multas que pueden superar los $3.000 millones. Un solo ataque de ransomware no solo significa una sanción regulatoria: significa perder la confianza de cada cliente que les confió su información.
-Resility funciona como tu equipo de ciberseguridad 24/7, sin que tengas que armar ni financiar uno interno. Nuestra IA, entrenada en amenazas reales de Latinoamérica, reduce el tiempo de detección de incidentes en un 70% frente a un SOC tradicional.
-¿Tienes 15 minutos esta semana para que te muestre cómo proteger Seguros Broker de forma concreta y sin complejidad?
-Quedo atenta a tu respuesta.
+          <t>Lily,
+Como corredora de seguros, Seguros Broker maneja a diario RUT, datos de salud, pólizas y cuentas bancarias de cientos de clientes. Información que los atacantes buscan activamente porque saben que las corredoras rara vez tienen un equipo de ciberseguridad dedicado.
+Con la Ley 21.663 ya vigente, una filtración no solo significa perder clientes y reputación — significa multas de hasta $3.000 millones CLP. Y la CMF está endureciendo las exigencias para intermediarios del mercado asegurador cada trimestre.
+Resility funciona como tu equipo de ciberseguridad 24/7 sin el costo de armar uno interno. Nuestra IA, entrenada en amenazas reales de Latinoamérica, reduce el tiempo de detección de incidentes en un 70% versus un SOC tradicional.
+¿Tienes 15 minutos esta semana para que te muestre cómo proteger a Seguros Broker antes de que sea obligatorio explicar por qué no lo hiciste?
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>
@@ -729,16 +729,16 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Alta Fe maneja datos sensibles de miles de asegurados — ¿quién los protege hoy?</t>
+          <t>Un ransomware cierra corredoras en 48 horas</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Juan, buenas tardes.
-Las corredoras de seguros como Alta Fe custodian información crítica de sus clientes: RUT, datos de salud, pólizas, siniestros y cuentas bancarias. Son exactamente el tipo de empresa que los atacantes buscan porque saben que no tienen un equipo de ciberseguridad dedicado.
-Con la Ley 21.663 ya vigente, la responsabilidad es directa: reportar incidentes es obligatorio y las multas llegan hasta $3.000 millones CLP. Un ransomware o una filtración no solo significa una sanción regulatoria, significa perder la confianza de cada cliente que les confió sus datos.
-Resility opera como tu equipo de ciberseguridad 24/7 sin que tengas que armar ni contratar uno. Nuestra IA detecta amenazas en menos de 15 minutos — un 70% más rápido que un SOC tradicional — y te mantiene en cumplimiento con CMF y la nueva ley.
-¿Tienes 15 minutos esta semana para una llamada rápida? Te muestro qué riesgos concretos enfrenta hoy Alta Fe y cómo resolverlos.
+          <t>Juan,
+Como corredora de seguros, Alta Fe maneja a diario RUTs, datos de salud, pólizas y cuentas bancarias de cientos de clientes. Es exactamente el tipo de información que los atacantes buscan, y las corredoras medianas son hoy el blanco preferido porque rara vez tienen un equipo de ciberseguridad dedicado.
+El problema es que ya no es opcional protegerse. La Ley 21.663 obliga a resguardar datos personales y reportar incidentes, con multas de hasta $3.000 millones CLP. Y la CMF está endureciendo las exigencias para intermediarios del mercado asegurador.
+En Resility operamos como tu equipo de ciberseguridad externo: monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio resuelto, sin que tengas que armar ni un cargo nuevo.
+¿Tienes 15 minutos esta semana para una llamada rápida? Te muestro en concreto qué riesgos tiene Alta Fe hoy y cómo cerrarlos.
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>
@@ -789,17 +789,17 @@
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Clan Seguros: datos de clientes expuestos sin equipo de ciberseguridad propio</t>
+          <t>Un ransomware cierra una corredora en 48h</t>
         </is>
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>Jorge, buenas tardes.
-Las corredoras de seguros como Clan manejan a diario RUT, datos de salud, pólizas y cuentas bancarias de cientos de clientes, y son exactamente el perfil que los atacantes eligen porque saben que no cuentan con un equipo de ciberseguridad dedicado.
-Con la Ley 21.663 ya vigente, una filtración o un ransomware no solo destruye la confianza de tus asegurados: implica multas de hasta $3.000 millones y obligación de reporte a la CMF.
-En Resility operamos como tu CyberSOC externo con IA, monitoreando 24/7 sin que necesites armar equipo ni invertir en infraestructura. Nuestros clientes del sector seguros reducen en un 70% el tiempo de detección de amenazas frente a un esquema tradicional.
-¿Tienes 15 minutos esta semana para mostrarte cómo proteger los datos de Clan de forma concreta y a un costo que hace sentido para una corredora?
-Quedo atento, Jorge.
+          <t>Jorge,
+Las corredoras de seguros manejan RUT, datos de salud, cuentas bancarias y siniestros de miles de personas, y son exactamente el tipo de empresa que los atacantes eligen porque saben que no tienen equipo de ciberseguridad propio.
+Con la Ley 21.663 ya vigente, Clan Corredores de Seguros está obligada a proteger esos datos y reportar incidentes bajo multas de hasta $3.000 millones. La pregunta no es si van a intentar atacarlos, sino cuándo.
+Resility opera como tu CyberSOC externo: monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio resuelto, sin que tengas que armar ni un solo cargo nuevo en tu equipo.
+Nuestros clientes reducen un 70% el tiempo de detección de ataques versus un esquema tradicional.
+¿Tienes 15 minutos esta semana para una llamada breve? Te muestro en concreto qué riesgos tiene hoy una corredora como Clan y cómo cerrarlos rápido.
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>
@@ -850,17 +850,16 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>MCA Chile: datos de asegurados expuestos sin equipo de ciberseguridad</t>
+          <t>¿Quién protege las pólizas de sus clientes hoy?</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
           <t>Berenguer,
-Las corredoras de seguros como MCA Chile manejan a diario RUT, datos de salud, pólizas y cuentas bancarias de cientos de clientes — y son exactamente el eslabón que los atacantes eligen para llegar a las aseguradoras. Sin un equipo de ciberseguridad dedicado, ese riesgo hoy es real y tiene consecuencias concretas.
-Con la Ley 21.663 vigente, una filtración o ransomware no solo destruye la confianza de tus clientes: implica multas de hasta $3.000 millones CLP y obligaciones de reporte que no se pueden improvisar.
-En Resility operamos como tu CyberSOC externalizado — monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio resuelto, sin que tengas que armar ni un solo cargo interno.
-Nuestros clientes reducen en un 70% el tiempo de detección de incidentes respecto a un esquema tradicional.
-¿Tienes 15 minutos esta semana para una llamada rápida? Me adapto a tu agenda.
+Las corredoras de seguros en Chile manejan RUT, datos de salud, cuentas bancarias y detalles de siniestros de miles de personas — y la mayoría no tiene un solo profesional dedicado a ciberseguridad. MCA Chile no es la excepción del mercado: es el blanco perfecto.
+La Ley 21.663 ya es realidad. Las multas llegan hasta $3.000 millones CLP, y los atacantes saben que las corredoras son la puerta más fácil hacia toda la cadena aseguradora.
+Resility opera como tu equipo de ciberseguridad 24/7 sin que tengas que armar uno. Nuestra IA, entrenada en amenazas de la región, detecta incidentes un 70% más rápido que un SOC tradicional — y responde en menos de 15 minutos.
+¿Tienes 15 minutos esta semana para que te muestre en concreto qué riesgos tiene hoy MCA Chile y cómo cerrarlos rápido?
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>
@@ -911,16 +910,17 @@
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>Cono Sur Seguros: datos de asegurados expuestos sin monitoreo 24/7</t>
+          <t>¿Quién protege los datos de sus asegurados hoy?</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
           <t>Roberto,
-Las corredoras de seguros como Cono Sur manejan a diario RUT, datos de salud, pólizas y cuentas bancarias de cientos de clientes. Son exactamente el tipo de empresa que los atacantes eligen como puerta de entrada al ecosistema asegurador, precisamente porque no cuentan con un equipo de ciberseguridad dedicado.
-Con la Ley 21.663 ya vigente, una filtración de datos no solo implica perder la confianza de tus asegurados: significa multas de hasta $3.000 millones CLP y obligación de reporte ante la autoridad.
-En Resility operamos como tu CyberSOC externalizado con IA, monitoreando amenazas 24/7 sin que necesites armar ni un solo cargo interno. Nuestros clientes del sector reducen en un 70% el tiempo de detección de incidentes versus un esquema tradicional.
-¿Tienes 15 minutos esta semana para que te muestre cómo proteger los datos de tus clientes antes de que sea un problema regulatorio?
+Las corredoras de seguros manejan RUT, datos de salud, información financiera y detalles de siniestros de cientos de clientes. Son exactamente el tipo de empresa que los atacantes buscan: datos valiosos y, generalmente, sin equipo de ciberseguridad dedicado.
+Con la Ley 21.663 ya vigente, Cono Sur Corredores de Seguros está obligada a proteger esa información y reportar incidentes, con multas que llegan hasta $3.000 millones. Y la CMF sigue endureciendo las exigencias para intermediarios del mercado asegurador.
+Resility funciona como tu equipo de ciberseguridad externo: monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio resuelto, sin que tengas que armar ni un cargo nuevo.
+Nuestros clientes del sector reducen un 70% el tiempo de detección de incidentes versus un esquema tradicional.
+¿Tienes 15 minutos esta semana para una llamada rápida? Te muestro qué riesgos concretos enfrenta hoy una corredora como la tuya.
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>
@@ -971,17 +971,16 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Phersu maneja datos sensibles de miles de asegurados — ¿quién los protege hoy?</t>
+          <t>¿Quién protege las pólizas de sus clientes hoy?</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
           <t>Cesar,
-Como corredora de seguros, Phersu custodia a diario información crítica de sus clientes: RUT, datos de salud, pólizas, siniestros, cuentas bancarias. Esa información es exactamente lo que buscan los atacantes, y las corredoras medianas son hoy el blanco preferido porque rara vez tienen un equipo de ciberseguridad dedicado.
-Con la Ley 21.663 ya vigente, una filtración de datos o un ransomware no solo paraliza la operación — implica multas de hasta $3.000 millones CLP y un daño reputacional difícil de revertir ante aseguradoras y clientes.
-Resility funciona como tu equipo de ciberseguridad externo: monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio resuelto, sin que tengas que contratar especialistas ni armar infraestructura.
-Nuestros clientes reducen un 70% el tiempo de detección de incidentes respecto a un esquema tradicional.
-¿Tienes 15 minutos esta semana para una llamada rápida? Me encantaría mostrarte cómo proteger a Phersu de forma simple y concreta.
+Las corredoras de seguros como Phersu manejan a diario RUT, datos de salud, cuentas bancarias y detalles de siniestros de cientos de clientes. Son exactamente el tipo de empresa que los atacantes buscan: datos valiosos y, generalmente, sin un equipo de ciberseguridad dedicado.
+Con la Ley 21.663 ya vigente, una filtración de datos no solo significa perder la confianza de sus asegurados — implica multas de hasta $3.000 millones CLP y la obligación de reportar incidentes públicamente.
+En Resility operamos como el equipo de ciberseguridad externo de corredoras y empresas del sector asegurador: monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio CMF — sin que usted tenga que armar ni un cargo nuevo.
+¿Tiene 15 minutos esta semana para revisar cómo se ve la exposición real de Phersu? Sin compromiso, solo diagnóstico.
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>
@@ -1032,16 +1031,17 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Oscar, datos de asegurados de Harder expuestos sin monitoreo es un riesgo que ya tiene multa</t>
+          <t>Una filtración de pólizas y no hay vuelta</t>
         </is>
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>Oscar,
-Las corredoras de seguros familiares como Oscar Harder e Hija custodian algo tremendamente valioso: RUT, datos de salud, información financiera y detalles de siniestros de cientos de clientes. Y en la gran mayoría de los casos, sin un solo recurso dedicado a ciberseguridad.
-Con la Ley 21.663 ya vigente, una filtración de datos o un ransomware no solo frena tu operación —implica multas de hasta $3.000 millones CLP y un daño reputacional que una corredora mediana difícilmente recupera. Los atacantes lo saben: buscan exactamente al eslabón menos protegido de la cadena aseguradora.
-Resility funciona como tu equipo de ciberseguridad 24/7 sin que tengas que armar ni contratar uno. Nuestra IA, entrenada en amenazas reales de Latinoamérica, detecta incidentes un 70% más rápido que un SOC tradicional y responde en menos de 15 minutos.
-¿Tienes 15 minutos esta semana para que te muestre cómo proteger los datos de tus asegurados sin complejidad?
+          <t>Oscar, buenas tardes.
+Las corredoras de seguros familiares como Oscar Harder e Hija manejan algo que los atacantes buscan activamente: RUT, datos de salud, cuentas bancarias y detalles de siniestros de cientos de clientes. Todo concentrado, y casi siempre sin un equipo de ciberseguridad dedicado.
+Desde 2024, la Ley 21.663 obliga a proteger esos datos y reportar incidentes, con multas que llegan a $3.000 millones CLP. Para una corredora mediana, una filtración no es solo una multa — es perder la confianza que llevan años construyendo.
+Resility funciona como tu equipo de ciberseguridad externo: monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio resuelto, sin que tengas que contratar especialistas.
+¿Tienes 15 minutos esta semana para revisar juntos qué tan expuesta está hoy la corredora? Sin compromiso, solo un diagnóstico claro.
+Quedo atento,
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>
@@ -1092,17 +1092,17 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>CP Brokers: datos de asegurados expuestos sin protección ante la nueva Ley de Ciberseguridad</t>
+          <t>Una filtración de pólizas y CP Brokers desaparece</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
           <t>Isidoro,
-Las corredoras de seguros como CP Brokers manejan a diario RUT, datos de salud, pólizas y cuentas bancarias de cientos de clientes, y hoy son el blanco preferido de los atacantes precisamente porque no cuentan con equipos de ciberseguridad propios. Los criminales lo saben y las usan como puerta de entrada a toda la cadena aseguradora.
-Con la Ley 21.663 ya vigente, una filtración o un ransomware no solo destruye la confianza de tus clientes: implica multas de hasta $3.000 millones y obligación de reporte ante la CMF.
-En Resility operamos como tu equipo de ciberseguridad externo, con monitoreo 24/7 potenciado por IA y respuesta en menos de 15 minutos ante incidentes críticos. Nuestros clientes del sector reducen un 70% el tiempo de detección de amenazas, sin el costo de armar un área interna.
-¿Tienes 15 minutos esta semana para mostrarte cómo proteger CP Brokers de forma concreta y rápida?
-Quedo atento,
+Las corredoras de seguros son hoy el blanco favorito de los atacantes en Chile. No por su tamaño, sino por lo que guardan: datos de salud, siniestros, RUT, cuentas bancarias de cientos de clientes. Y la mayoría no tiene ni una persona dedicada a ciberseguridad.
+Con la Ley 21.663 ya vigente, una brecha de datos puede significar multas de hasta $3.000 millones CLP, además del daño reputacional que ninguna póliza cubre.
+En Resility operamos como el equipo de ciberseguridad externo de empresas como CP Brokers: monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio CMF — sin que tengas que armar ni un cargo nuevo.
+Nuestros clientes reducen en un 70% el tiempo de detección de incidentes respecto a un esquema tradicional.
+¿Tienes 15 minutos esta semana para una conversación rápida? Me adapto a tu agenda.
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Add LinkedIn verification step before email generation
New verify_linkedin() searches DuckDuckGo for each contact's
name + company + linkedin filtered to 2025/2026. Returns
"✅ Verificado" or "⚠️ Verificar manualmente". Column added
to Excel with color-coded cells (green/yellow).

https://claude.ai/code/session_01DWU7frtt2nZeg1H9Fnsb63
</commit_message>
<xml_diff>
--- a/resility_correos_corredoras.xlsx
+++ b/resility_correos_corredoras.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,8 +41,13 @@
       <name val="Calibri"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="0092400E"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -62,6 +67,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -96,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -113,13 +123,16 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -487,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -501,12 +514,13 @@
     <col width="40" customWidth="1" min="9" max="9"/>
     <col width="70" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RESILITY — Correos de Ventas Personalizados  |  Generado: 12/03/2026 19:56</t>
+          <t>RESILITY — Correos de Ventas Personalizados  |  Generado: 12/03/2026 20:28</t>
         </is>
       </c>
     </row>
@@ -564,6 +578,11 @@
       <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Estado</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Verificación LinkedIn</t>
         </is>
       </c>
     </row>
@@ -608,83 +627,93 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>¿Quién protege las pólizas de sus clientes hoy?</t>
+          <t>¿Quién protege las pólizas y datos de sus asegurados?</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
           <t>María Isabel,
-Las corredoras de seguros son hoy el blanco favorito de los atacantes: manejan RUT, datos de salud, cuentas bancarias y detalles de siniestros de cientos de clientes, y rara vez cuentan con un equipo dedicado de ciberseguridad. Beroiza Seguros no es la excepción en ese perfil de riesgo.
-Con la Ley 21.663 ya vigente, una filtración de datos no solo destruye la confianza de sus asegurados — implica multas de hasta $3.000 millones CLP y la obligación de reportar incidentes ante la CMF.
-Resility actúa como su equipo de ciberseguridad 24/7, sin que necesite contratar ni un solo especialista. Nuestra IA, entrenada en amenazas reales de Latinoamérica, reduce el tiempo de detección de incidentes en un 70% versus un SOC tradicional.
-¿Tiene 15 minutos esta semana para que le muestre qué tan expuesta está su operación hoy y cómo cerramos esas brechas rápidamente?
-Quedo atenta a su respuesta.
+Las corredoras de seguros manejan lo más sensible que existe: datos de salud, RUT, cuentas bancarias y detalles de siniestros de cientos de clientes. Y en la mayoría de los casos, no tienen a nadie dedicado a proteger esa información.
+Con la Ley 21.663 ya vigente, una filtración o ataque ransomware no solo destruye la confianza de sus asegurados — implica multas de hasta $3.000 millones. Los atacantes lo saben y apuntan al eslabón que menos invierte en defensa: las corredoras.
+Resility actúa como el equipo de ciberseguridad que Beroiza Seguros necesita, sin el costo de armarlo internamente. Monitoreamos 24/7 con inteligencia artificial entrenada en amenazas reales de Chile y LATAM, reduciendo en un 70% el tiempo de detección frente a un incidente.
+¿Podemos conversar 15 minutos esta semana? Le muestro en concreto qué riesgos tiene hoy y cómo cerrarlos rápido.
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ Verificar manualmente</t>
         </is>
       </c>
     </row>
     <row r="4" ht="120" customHeight="1">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Lily Justiniano</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Gerente General</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>Seguros Broker Corredores de Seguros</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>Corredora de Seguros</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>ljustiniano@segurosbroker.cl</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>+56 9 8819457</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>https://www.segurosbroker.cl</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr">
-        <is>
-          <t>¿Quién protege los datos de sus asegurados hoy?</t>
-        </is>
-      </c>
-      <c r="J4" s="8" t="inlineStr">
-        <is>
-          <t>Lily,
-Como corredora de seguros, Seguros Broker maneja a diario RUT, datos de salud, pólizas y cuentas bancarias de cientos de clientes. Información que los atacantes buscan activamente porque saben que las corredoras rara vez tienen un equipo de ciberseguridad dedicado.
-Con la Ley 21.663 ya vigente, una filtración no solo significa perder clientes y reputación — significa multas de hasta $3.000 millones CLP. Y la CMF está endureciendo las exigencias para intermediarios del mercado asegurador cada trimestre.
-Resility funciona como tu equipo de ciberseguridad 24/7 sin el costo de armar uno interno. Nuestra IA, entrenada en amenazas reales de Latinoamérica, reduce el tiempo de detección de incidentes en un 70% versus un SOC tradicional.
-¿Tienes 15 minutos esta semana para que te muestre cómo proteger a Seguros Broker antes de que sea obligatorio explicar por qué no lo hiciste?
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Datos de pólizas expuestos sin que lo sepan</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>Lily, buenas tardes.
+Las corredoras de seguros manejan RUT, datos de salud, cuentas bancarias y detalle de siniestros de cientos de clientes — y en la mayoría de los casos, no hay nadie vigilando esa información 24/7.
+Esto ya no es solo un riesgo operacional. La Ley 21.663 obliga a empresas como Seguros Broker a proteger datos personales y reportar incidentes, con multas que llegan hasta $3.000 millones. Y los atacantes lo saben: las corredoras son el eslabón más fácil para entrar a toda la cadena aseguradora.
+Resility funciona como tu equipo de ciberseguridad completo, sin el costo de armar uno interno. Monitoreamos con IA 24/7 y respondemos en menos de 15 minutos ante cualquier incidente crítico — reduciendo un 70% el tiempo de detección versus un esquema tradicional.
+¿Tienes 15 minutos esta semana para que te muestre cómo proteger la operación de Seguros Broker de forma concreta?
+Quedo atenta a tu respuesta.
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="K4" s="7" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ Verificar manualmente</t>
         </is>
       </c>
     </row>
@@ -735,77 +764,86 @@
       <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Juan,
-Como corredora de seguros, Alta Fe maneja a diario RUTs, datos de salud, pólizas y cuentas bancarias de cientos de clientes. Es exactamente el tipo de información que los atacantes buscan, y las corredoras medianas son hoy el blanco preferido porque rara vez tienen un equipo de ciberseguridad dedicado.
-El problema es que ya no es opcional protegerse. La Ley 21.663 obliga a resguardar datos personales y reportar incidentes, con multas de hasta $3.000 millones CLP. Y la CMF está endureciendo las exigencias para intermediarios del mercado asegurador.
-En Resility operamos como tu equipo de ciberseguridad externo: monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio resuelto, sin que tengas que armar ni un cargo nuevo.
-¿Tienes 15 minutos esta semana para una llamada rápida? Te muestro en concreto qué riesgos tiene Alta Fe hoy y cómo cerrarlos.
+Como corredora de seguros, Alta Fe maneja a diario RUT, datos de salud, pólizas y cuentas bancarias de cientos de clientes. Esa información es exactamente lo que buscan los atacantes, y las corredoras son hoy el eslabón más vulnerable de la cadena aseguradora.
+La Ley 21.663 ya es una realidad: obliga a reportar incidentes y proteger datos personales, con multas de hasta $3.000 millones CLP. La pregunta es directa: ¿quién está vigilando hoy la seguridad de esa información en Alta Fe?
+En Resility operamos como tu equipo de ciberseguridad 24/7, sin que tengas que armar ni un cargo interno. Nuestra IA detecta amenazas en menos de 15 minutos, un 70% más rápido que un SOC tradicional.
+¿Tienes 15 minutos esta semana para una llamada? Te muestro en concreto qué riesgos tiene una corredora como Alta Fe hoy y cómo cerrarlos rápido.
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ Verificar manualmente</t>
         </is>
       </c>
     </row>
     <row r="6" ht="120" customHeight="1">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Jorge Urtuvia</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Gerente General</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>Clan Corredores de Seguros</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Corredora de Seguros</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>jurtuvia@clanseguros.cl</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>+56 9 6125104</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>https://www.clanseguros.cl</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr">
-        <is>
-          <t>Un ransomware cierra una corredora en 48h</t>
-        </is>
-      </c>
-      <c r="J6" s="8" t="inlineStr">
-        <is>
-          <t>Jorge,
-Las corredoras de seguros manejan RUT, datos de salud, cuentas bancarias y siniestros de miles de personas, y son exactamente el tipo de empresa que los atacantes eligen porque saben que no tienen equipo de ciberseguridad propio.
-Con la Ley 21.663 ya vigente, Clan Corredores de Seguros está obligada a proteger esos datos y reportar incidentes bajo multas de hasta $3.000 millones. La pregunta no es si van a intentar atacarlos, sino cuándo.
-Resility opera como tu CyberSOC externo: monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio resuelto, sin que tengas que armar ni un solo cargo nuevo en tu equipo.
-Nuestros clientes reducen un 70% el tiempo de detección de ataques versus un esquema tradicional.
-¿Tienes 15 minutos esta semana para una llamada breve? Te muestro en concreto qué riesgos tiene hoy una corredora como Clan y cómo cerrarlos rápido.
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>¿Quién protege las pólizas de sus clientes hoy?</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>Jorge, buenas tardes.
+Las corredoras de seguros como Clan manejan algo que los atacantes buscan activamente: RUT, datos de salud, información financiera y detalles de siniestros de cientos de clientes. Todo concentrado, y en la mayoría de los casos, sin un equipo de ciberseguridad dedicado.
+Esto ya no es solo un riesgo operacional. La Ley 21.663 obliga a reportar incidentes y proteger datos personales, con multas de hasta $3.000 millones CLP. Y la CMF está endureciendo las exigencias para intermediarios del mercado asegurador cada trimestre.
+Resility funciona como tu equipo de ciberseguridad externo: monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio resuelto — sin que tengas que armar ni un cargo nuevo.
+¿Tienes 15 minutos esta semana para una conversación rápida? Te muestro en concreto qué riesgos tiene Clan hoy y cómo cerrarlos.
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr">
+      <c r="K6" s="7" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ Verificar manualmente</t>
         </is>
       </c>
     </row>
@@ -856,77 +894,87 @@
       <c r="J7" s="5" t="inlineStr">
         <is>
           <t>Berenguer,
-Las corredoras de seguros en Chile manejan RUT, datos de salud, cuentas bancarias y detalles de siniestros de miles de personas — y la mayoría no tiene un solo profesional dedicado a ciberseguridad. MCA Chile no es la excepción del mercado: es el blanco perfecto.
-La Ley 21.663 ya es realidad. Las multas llegan hasta $3.000 millones CLP, y los atacantes saben que las corredoras son la puerta más fácil hacia toda la cadena aseguradora.
-Resility opera como tu equipo de ciberseguridad 24/7 sin que tengas que armar uno. Nuestra IA, entrenada en amenazas de la región, detecta incidentes un 70% más rápido que un SOC tradicional — y responde en menos de 15 minutos.
-¿Tienes 15 minutos esta semana para que te muestre en concreto qué riesgos tiene hoy MCA Chile y cómo cerrarlos rápido?
+Las corredoras de seguros son hoy el blanco preferido de los ciberataques en Chile. Manejan RUT, datos de salud, siniestros y cuentas bancarias de miles de personas, y generalmente no cuentan con un equipo dedicado de ciberseguridad. MCA Chile calza exactamente en ese perfil de riesgo.
+Con la Ley 21.663 ya vigente, una filtración de datos no solo destruye la confianza de sus asegurados — implica multas de hasta $3.000 millones CLP.
+En Resility operamos como su equipo de ciberseguridad externo: monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio ante la CMF. Sin que usted tenga que armar ni un cargo nuevo.
+Nuestros clientes reducen en un 70% el tiempo de detección de incidentes versus un esquema tradicional.
+¿Tiene 15 minutos esta semana para una conversación breve? Le muestro en concreto qué riesgos tiene hoy MCA Chile y cómo cerrarlos rápido.
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ Verificar manualmente</t>
         </is>
       </c>
     </row>
     <row r="8" ht="120" customHeight="1">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Roberto Gatica</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Gerente</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Cono Sur Corredores de Seguros</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>Corredora de Seguros</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>roberto.gatica@conosurseguros.cl</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>+56 9 1294214</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>https://www.conosurseguros.cl</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>¿Quién protege los datos de sus asegurados hoy?</t>
         </is>
       </c>
-      <c r="J8" s="8" t="inlineStr">
+      <c r="J8" s="9" t="inlineStr">
         <is>
           <t>Roberto,
-Las corredoras de seguros manejan RUT, datos de salud, información financiera y detalles de siniestros de cientos de clientes. Son exactamente el tipo de empresa que los atacantes buscan: datos valiosos y, generalmente, sin equipo de ciberseguridad dedicado.
-Con la Ley 21.663 ya vigente, Cono Sur Corredores de Seguros está obligada a proteger esa información y reportar incidentes, con multas que llegan hasta $3.000 millones. Y la CMF sigue endureciendo las exigencias para intermediarios del mercado asegurador.
-Resility funciona como tu equipo de ciberseguridad externo: monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio resuelto, sin que tengas que armar ni un cargo nuevo.
-Nuestros clientes del sector reducen un 70% el tiempo de detección de incidentes versus un esquema tradicional.
-¿Tienes 15 minutos esta semana para una llamada rápida? Te muestro qué riesgos concretos enfrenta hoy una corredora como la tuya.
+Las corredoras de seguros manejan lo más sensible que existe: datos de salud, RUT, información financiera y siniestros de cientos de clientes. Y en la gran mayoría, no hay nadie vigilando esa información 24/7.
+Con la Ley 21.663 ya vigente, Cono Sur Corredores de Seguros está obligada a proteger esos datos y reportar incidentes — con multas que llegan a $3.000 millones. Los atacantes lo saben: las corredoras son el eslabón más fácil para entrar a toda la cadena aseguradora.
+En Resility operamos como tu equipo de ciberseguridad completo, sin que tengas que armar uno interno. Nuestro CyberSOC con IA monitorea tu operación 24/7 y responde en menos de 15 minutos ante cualquier incidente crítico — reduciendo un 70% el tiempo de detección versus un esquema tradicional.
+¿Tienes 15 minutos esta semana para revisarlo? Te muestro en concreto qué riesgos tiene hoy una corredora como la tuya y cómo cerrarlos rápido.
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="K8" s="7" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ Verificar manualmente</t>
         </is>
       </c>
     </row>
@@ -971,83 +1019,93 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>¿Quién protege las pólizas de sus clientes hoy?</t>
+          <t>¿Quién protege los datos sensibles de Phersu hoy?</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
           <t>Cesar,
-Las corredoras de seguros como Phersu manejan a diario RUT, datos de salud, cuentas bancarias y detalles de siniestros de cientos de clientes. Son exactamente el tipo de empresa que los atacantes buscan: datos valiosos y, generalmente, sin un equipo de ciberseguridad dedicado.
-Con la Ley 21.663 ya vigente, una filtración de datos no solo significa perder la confianza de sus asegurados — implica multas de hasta $3.000 millones CLP y la obligación de reportar incidentes públicamente.
-En Resility operamos como el equipo de ciberseguridad externo de corredoras y empresas del sector asegurador: monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio CMF — sin que usted tenga que armar ni un cargo nuevo.
-¿Tiene 15 minutos esta semana para revisar cómo se ve la exposición real de Phersu? Sin compromiso, solo diagnóstico.
+Las corredoras de seguros son hoy el blanco favorito de los ciberataques en Chile. Manejan RUT, datos de salud, pólizas y cuentas bancarias de cientos de clientes — y la mayoría no tiene un solo especialista en ciberseguridad dedicado.
+Con la Ley 21.663 vigente, Phersu está obligada a proteger esa información y reportar incidentes. Las multas llegan hasta $3.000 millones CLP. Un ransomware no solo paraliza la operación: destruye la confianza que tus asegurados depositaron en ustedes.
+Resility funciona como tu equipo de ciberseguridad completo, sin que tengas que armar uno. Monitoreamos tu infraestructura 24/7 con inteligencia artificial y respondemos en menos de 15 minutos ante un incidente crítico — reduciendo en un 70% el tiempo de detección versus un esquema tradicional.
+¿Tienes 15 minutos esta semana para revisar juntos tu nivel de exposición actual?
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ Verificar manualmente</t>
         </is>
       </c>
     </row>
     <row r="10" ht="120" customHeight="1">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Oscar Harder</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Gerente</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>Oscar Harder e Hija Corredores de Seguros</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>Corredora de Seguros</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>oficina@segurosharder.cl</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>+56 9 9161735</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>https://www.segurosharder.cl</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr">
-        <is>
-          <t>Una filtración de pólizas y no hay vuelta</t>
-        </is>
-      </c>
-      <c r="J10" s="8" t="inlineStr">
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Una filtración de pólizas y no hay vuelta atrás</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
         <is>
           <t>Oscar, buenas tardes.
-Las corredoras de seguros familiares como Oscar Harder e Hija manejan algo que los atacantes buscan activamente: RUT, datos de salud, cuentas bancarias y detalles de siniestros de cientos de clientes. Todo concentrado, y casi siempre sin un equipo de ciberseguridad dedicado.
-Desde 2024, la Ley 21.663 obliga a proteger esos datos y reportar incidentes, con multas que llegan a $3.000 millones CLP. Para una corredora mediana, una filtración no es solo una multa — es perder la confianza que llevan años construyendo.
-Resility funciona como tu equipo de ciberseguridad externo: monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio resuelto, sin que tengas que contratar especialistas.
-¿Tienes 15 minutos esta semana para revisar juntos qué tan expuesta está hoy la corredora? Sin compromiso, solo un diagnóstico claro.
-Quedo atento,
+Las corredoras de seguros familiares como Oscar Harder e Hija manejan algo que los atacantes buscan activamente: RUT, datos de salud, información financiera y detalle de siniestros de cientos de clientes. Todo concentrado, y generalmente sin un equipo de ciberseguridad dedicado.
+Con la Ley 21.663 ya vigente, una filtración no solo significa perder la confianza que han construido por años — significa multas de hasta $3.000 millones CLP y obligación de reportar públicamente el incidente.
+Resility funciona como tu equipo de ciberseguridad externo: monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio resuelto. Sin contratar personal ni armar infraestructura.
+Nuestros clientes del sector seguros redujeron un 70% el tiempo de exposición a amenazas desde el primer mes.
+¿Tienes 15 minutos esta semana para una llamada breve? Me adapto a tu agenda.
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>
-      <c r="K10" s="6" t="inlineStr">
+      <c r="K10" s="7" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ Verificar manualmente</t>
         </is>
       </c>
     </row>
@@ -1098,23 +1156,27 @@
       <c r="J11" s="5" t="inlineStr">
         <is>
           <t>Isidoro,
-Las corredoras de seguros son hoy el blanco favorito de los atacantes en Chile. No por su tamaño, sino por lo que guardan: datos de salud, siniestros, RUT, cuentas bancarias de cientos de clientes. Y la mayoría no tiene ni una persona dedicada a ciberseguridad.
-Con la Ley 21.663 ya vigente, una brecha de datos puede significar multas de hasta $3.000 millones CLP, además del daño reputacional que ninguna póliza cubre.
-En Resility operamos como el equipo de ciberseguridad externo de empresas como CP Brokers: monitoreo 24/7 con inteligencia artificial, detección de amenazas en menos de 15 minutos y cumplimiento regulatorio CMF — sin que tengas que armar ni un cargo nuevo.
-Nuestros clientes reducen en un 70% el tiempo de detección de incidentes respecto a un esquema tradicional.
-¿Tienes 15 minutos esta semana para una conversación rápida? Me adapto a tu agenda.
+Las corredoras de seguros son hoy el blanco favorito de los atacantes en Chile. Manejan RUT, datos de salud, siniestros y cuentas bancarias de miles de personas, pero rara vez cuentan con un equipo dedicado de ciberseguridad. CP Brokers tiene exactamente ese perfil de riesgo.
+Con la Ley 21.663 ya vigente, una brecha de datos no solo destruye la confianza de tus clientes — implica multas de hasta $3.000 millones CLP y la obligación de reportar incidentes que hoy probablemente nadie en tu equipo sabría gestionar.
+Resility funciona como tu equipo de ciberseguridad externo, con monitoreo 24/7 e inteligencia artificial, sin que necesites contratar ni una persona. Nuestros clientes del sector asegurador reducen un 70% el tiempo de detección de amenazas versus un esquema tradicional.
+¿Tienes 15 minutos esta semana para una conversación rápida? Te muestro en concreto qué riesgos tiene hoy CP Brokers y cómo cerrarlos.
 Equipo Comercial, Resility | CyberSOC con IA</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ Verificar manualmente</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>